<commit_message>
adaptive mutate, plus, diversity penatly
</commit_message>
<xml_diff>
--- a/main/model_excel/analysis_results_0.6_0.9.xlsx
+++ b/main/model_excel/analysis_results_0.6_0.9.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cchih\Desktop\NTHU\MasterThesis\GA\SGM_GA\printing\regression\training_error_results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cchih\Desktop\NTHU\MasterThesis\GA\SGM_GA\main\model_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BC9DB2C-C9CA-4BB3-ABB5-1B28F481289A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C944B932-BFD0-4866-9348-7E765B97CA69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="17">
   <si>
     <t>Design_s1(mm)</t>
   </si>
@@ -569,17 +569,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="6" width="18.75" bestFit="1" customWidth="1"/>
     <col min="7" max="9" width="15.5" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="14.25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -613,17 +611,8 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:23">
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2">
         <v>0.6</v>
       </c>
@@ -657,36 +646,8 @@
       <c r="K2">
         <v>0.21254331848455779</v>
       </c>
-      <c r="L2">
-        <v>74</v>
-      </c>
-      <c r="M2">
-        <v>80.3</v>
-      </c>
-      <c r="N2">
-        <v>75.3</v>
-      </c>
-      <c r="P2" s="4">
-        <f>AVERAGE(L2:O2)</f>
-        <v>76.533333333333346</v>
-      </c>
-      <c r="Q2" s="6">
-        <f>P2/22</f>
-        <v>3.4787878787878794</v>
-      </c>
-      <c r="R2">
-        <v>60</v>
-      </c>
-      <c r="V2">
-        <f>AVERAGE(R2:U2)</f>
-        <v>60</v>
-      </c>
-      <c r="W2" s="6">
-        <f>V2/22</f>
-        <v>2.7272727272727271</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23">
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3">
         <v>0.6</v>
       </c>
@@ -720,45 +681,8 @@
       <c r="K3">
         <v>0.19708812999417119</v>
       </c>
-      <c r="L3">
-        <v>59.5</v>
-      </c>
-      <c r="M3">
-        <v>54.1</v>
-      </c>
-      <c r="N3">
-        <v>58.1</v>
-      </c>
-      <c r="O3">
-        <v>54.4</v>
-      </c>
-      <c r="P3" s="4">
-        <f t="shared" ref="P3:P11" si="0">AVERAGE(L3:O3)</f>
-        <v>56.524999999999999</v>
-      </c>
-      <c r="Q3" s="6">
-        <f t="shared" ref="Q3:Q11" si="1">P3/22</f>
-        <v>2.5693181818181818</v>
-      </c>
-      <c r="R3">
-        <v>39</v>
-      </c>
-      <c r="S3">
-        <v>49.1</v>
-      </c>
-      <c r="T3">
-        <v>46.9</v>
-      </c>
-      <c r="V3">
-        <f t="shared" ref="V3:V13" si="2">AVERAGE(R3:U3)</f>
-        <v>45</v>
-      </c>
-      <c r="W3" s="6">
-        <f>V3/22</f>
-        <v>2.0454545454545454</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23">
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4">
         <v>0.6</v>
       </c>
@@ -792,18 +716,8 @@
       <c r="K4">
         <v>0.2119764435925153</v>
       </c>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="6"/>
-      <c r="R4">
-        <v>49.1</v>
-      </c>
-      <c r="V4">
-        <f t="shared" si="2"/>
-        <v>49.1</v>
-      </c>
-      <c r="W4" s="6"/>
-    </row>
-    <row r="5" spans="1:23">
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5">
         <v>0.6</v>
       </c>
@@ -837,27 +751,8 @@
       <c r="K5">
         <v>0.44368714981957491</v>
       </c>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="6"/>
-      <c r="R5">
-        <v>35.5</v>
-      </c>
-      <c r="S5">
-        <v>33.299999999999997</v>
-      </c>
-      <c r="T5">
-        <v>39.200000000000003</v>
-      </c>
-      <c r="U5">
-        <v>38</v>
-      </c>
-      <c r="V5">
-        <f t="shared" si="2"/>
-        <v>36.5</v>
-      </c>
-      <c r="W5" s="6"/>
-    </row>
-    <row r="6" spans="1:23">
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6">
         <v>0.6</v>
       </c>
@@ -891,42 +786,8 @@
       <c r="K6">
         <v>0.26643957163933391</v>
       </c>
-      <c r="L6">
-        <v>48.4</v>
-      </c>
-      <c r="M6">
-        <v>48.1</v>
-      </c>
-      <c r="N6">
-        <v>51.1</v>
-      </c>
-      <c r="O6">
-        <v>50.1</v>
-      </c>
-      <c r="P6" s="4">
-        <f t="shared" si="0"/>
-        <v>49.424999999999997</v>
-      </c>
-      <c r="Q6" s="6">
-        <f t="shared" si="1"/>
-        <v>2.2465909090909091</v>
-      </c>
-      <c r="R6">
-        <v>28.8</v>
-      </c>
-      <c r="S6">
-        <v>30</v>
-      </c>
-      <c r="V6">
-        <f t="shared" si="2"/>
-        <v>29.4</v>
-      </c>
-      <c r="W6" s="6">
-        <f>V6/22</f>
-        <v>1.3363636363636362</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23">
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7">
         <v>0.6</v>
       </c>
@@ -960,26 +821,8 @@
       <c r="K7">
         <v>0.22478913777023921</v>
       </c>
-      <c r="L7">
-        <v>59.2</v>
-      </c>
-      <c r="M7">
-        <v>59.7</v>
-      </c>
-      <c r="N7">
-        <v>56.8</v>
-      </c>
-      <c r="P7" s="4">
-        <f t="shared" si="0"/>
-        <v>58.566666666666663</v>
-      </c>
-      <c r="Q7" s="6">
-        <f t="shared" si="1"/>
-        <v>2.6621212121212121</v>
-      </c>
-      <c r="W7" s="6"/>
-    </row>
-    <row r="8" spans="1:23">
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8">
         <v>0.9</v>
       </c>
@@ -1013,36 +856,8 @@
       <c r="K8">
         <v>8.2782325865386544E-2</v>
       </c>
-      <c r="L8">
-        <v>71.900000000000006</v>
-      </c>
-      <c r="M8">
-        <v>71.5</v>
-      </c>
-      <c r="N8">
-        <v>72</v>
-      </c>
-      <c r="P8" s="4">
-        <f t="shared" si="0"/>
-        <v>71.8</v>
-      </c>
-      <c r="Q8" s="6">
-        <f t="shared" si="1"/>
-        <v>3.2636363636363637</v>
-      </c>
-      <c r="R8">
-        <v>77.5</v>
-      </c>
-      <c r="V8">
-        <f t="shared" si="2"/>
-        <v>77.5</v>
-      </c>
-      <c r="W8" s="6">
-        <f t="shared" ref="W8:W12" si="3">V8/22</f>
-        <v>3.5227272727272729</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23">
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9">
         <v>0.9</v>
       </c>
@@ -1076,48 +891,8 @@
       <c r="K9">
         <v>0.1149392607649912</v>
       </c>
-      <c r="L9">
-        <v>56.6</v>
-      </c>
-      <c r="M9">
-        <v>52.3</v>
-      </c>
-      <c r="N9">
-        <v>51.4</v>
-      </c>
-      <c r="O9">
-        <v>49.3</v>
-      </c>
-      <c r="P9" s="4">
-        <f t="shared" si="0"/>
-        <v>52.400000000000006</v>
-      </c>
-      <c r="Q9" s="6">
-        <f t="shared" si="1"/>
-        <v>2.3818181818181823</v>
-      </c>
-      <c r="R9">
-        <v>34.200000000000003</v>
-      </c>
-      <c r="S9">
-        <v>40.200000000000003</v>
-      </c>
-      <c r="T9">
-        <v>32.9</v>
-      </c>
-      <c r="U9">
-        <v>33.700000000000003</v>
-      </c>
-      <c r="V9">
-        <f t="shared" si="2"/>
-        <v>35.25</v>
-      </c>
-      <c r="W9" s="6">
-        <f t="shared" si="3"/>
-        <v>1.6022727272727273</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23">
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10">
         <v>0.9</v>
       </c>
@@ -1151,21 +926,8 @@
       <c r="K10">
         <v>0.1280036144376335</v>
       </c>
-      <c r="P10" s="4"/>
-      <c r="Q10" s="6"/>
-      <c r="R10">
-        <v>32.4</v>
-      </c>
-      <c r="S10">
-        <v>35.700000000000003</v>
-      </c>
-      <c r="V10">
-        <f t="shared" si="2"/>
-        <v>34.049999999999997</v>
-      </c>
-      <c r="W10" s="6"/>
-    </row>
-    <row r="11" spans="1:23">
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11">
         <v>0.9</v>
       </c>
@@ -1199,42 +961,8 @@
       <c r="K11">
         <v>0.13348512174602031</v>
       </c>
-      <c r="L11">
-        <v>51.6</v>
-      </c>
-      <c r="M11">
-        <v>53.9</v>
-      </c>
-      <c r="N11">
-        <v>53.2</v>
-      </c>
-      <c r="O11">
-        <v>55.4</v>
-      </c>
-      <c r="P11" s="4">
-        <f t="shared" si="0"/>
-        <v>53.524999999999999</v>
-      </c>
-      <c r="Q11" s="6">
-        <f t="shared" si="1"/>
-        <v>2.4329545454545456</v>
-      </c>
-      <c r="R11">
-        <v>33.5</v>
-      </c>
-      <c r="S11">
-        <v>33.799999999999997</v>
-      </c>
-      <c r="V11">
-        <f t="shared" si="2"/>
-        <v>33.65</v>
-      </c>
-      <c r="W11" s="6">
-        <f t="shared" si="3"/>
-        <v>1.5295454545454545</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23">
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12">
         <v>0.9</v>
       </c>
@@ -1268,42 +996,8 @@
       <c r="K12">
         <v>0.13460192015497621</v>
       </c>
-      <c r="L12">
-        <v>47.3</v>
-      </c>
-      <c r="M12">
-        <v>47.7</v>
-      </c>
-      <c r="N12">
-        <v>46</v>
-      </c>
-      <c r="O12">
-        <v>47.3</v>
-      </c>
-      <c r="P12" s="4"/>
-      <c r="Q12" s="7"/>
-      <c r="R12">
-        <v>33.299999999999997</v>
-      </c>
-      <c r="S12">
-        <v>29.2</v>
-      </c>
-      <c r="T12">
-        <v>30</v>
-      </c>
-      <c r="U12">
-        <v>32</v>
-      </c>
-      <c r="V12">
-        <f t="shared" si="2"/>
-        <v>31.125</v>
-      </c>
-      <c r="W12" s="6">
-        <f t="shared" si="3"/>
-        <v>1.4147727272727273</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23">
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13">
         <v>0.9</v>
       </c>
@@ -1336,19 +1030,6 @@
       </c>
       <c r="K13">
         <v>0.13293458342743</v>
-      </c>
-      <c r="P13" s="4"/>
-      <c r="Q13" s="7"/>
-      <c r="R13">
-        <v>36.200000000000003</v>
-      </c>
-      <c r="V13">
-        <f t="shared" si="2"/>
-        <v>36.200000000000003</v>
-      </c>
-      <c r="W13" s="6">
-        <f>V13/22</f>
-        <v>1.6454545454545455</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mutation clip, add  crossover
</commit_message>
<xml_diff>
--- a/main/model_excel/analysis_results_0.6_0.9.xlsx
+++ b/main/model_excel/analysis_results_0.6_0.9.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cchih\Desktop\NTHU\MasterThesis\GA\SGM_GA\main\model_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F6F7CA8-A86D-46B0-93DB-D658762C9EE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16B9B378-322A-47DD-BC3F-302EFDDD9DEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="20">
   <si>
     <t>Design_s1(mm)</t>
   </si>
@@ -93,6 +93,18 @@
   </si>
   <si>
     <t>Rvally_px</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rv</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rt</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rvally_avg(um)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -569,7 +581,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="6" width="18.75" bestFit="1" customWidth="1"/>
@@ -577,7 +589,7 @@
     <col min="10" max="11" width="14.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -611,8 +623,14 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11">
+      <c r="L1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2">
         <v>0.6</v>
       </c>
@@ -647,7 +665,7 @@
         <v>0.21254331848455779</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:13">
       <c r="A3">
         <v>0.6</v>
       </c>
@@ -682,7 +700,7 @@
         <v>0.19708812999417119</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:13">
       <c r="A4">
         <v>0.6</v>
       </c>
@@ -717,7 +735,7 @@
         <v>0.2119764435925153</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:13">
       <c r="A5">
         <v>0.6</v>
       </c>
@@ -752,7 +770,7 @@
         <v>0.44368714981957491</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:13">
       <c r="A6">
         <v>0.6</v>
       </c>
@@ -787,7 +805,7 @@
         <v>0.26643957163933391</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:13">
       <c r="A7">
         <v>0.6</v>
       </c>
@@ -822,7 +840,7 @@
         <v>0.22478913777023921</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:13">
       <c r="A8">
         <v>0.9</v>
       </c>
@@ -857,7 +875,7 @@
         <v>8.2782325865386544E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:13">
       <c r="A9">
         <v>0.9</v>
       </c>
@@ -892,7 +910,7 @@
         <v>0.1149392607649912</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:13">
       <c r="A10">
         <v>0.9</v>
       </c>
@@ -927,7 +945,7 @@
         <v>0.1280036144376335</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:13">
       <c r="A11">
         <v>0.9</v>
       </c>
@@ -962,7 +980,7 @@
         <v>0.13348512174602031</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:13">
       <c r="A12">
         <v>0.9</v>
       </c>
@@ -997,7 +1015,7 @@
         <v>0.13460192015497621</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:13">
       <c r="A13">
         <v>0.9</v>
       </c>
@@ -1830,22 +1848,24 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8769C09C-C53B-4D4E-B105-51033AAB2610}">
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="6" width="18.75" bestFit="1" customWidth="1"/>
     <col min="7" max="9" width="15.5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.625" hidden="1" customWidth="1"/>
-    <col min="12" max="13" width="0" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="8.625" customWidth="1"/>
+    <col min="12" max="13" width="9" customWidth="1"/>
     <col min="14" max="14" width="15.125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.875" bestFit="1" customWidth="1"/>
-    <col min="17" max="19" width="0" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="13.75" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.875" bestFit="1" customWidth="1"/>
+    <col min="18" max="20" width="0" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="13.75" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.75" customWidth="1"/>
+    <col min="23" max="23" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:23">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1882,23 +1902,27 @@
       <c r="N1" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="14" t="s">
+      <c r="O1" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="P1" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="P1" s="14" t="s">
+      <c r="Q1" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="Q1" s="15"/>
       <c r="R1" s="15"/>
       <c r="S1" s="15"/>
-      <c r="T1" s="17" t="s">
+      <c r="T1" s="15"/>
+      <c r="U1" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="U1" s="17" t="s">
+      <c r="V1" s="17"/>
+      <c r="W1" s="17" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:21">
+    <row r="2" spans="1:23">
       <c r="A2" s="5">
         <v>0.6</v>
       </c>
@@ -1939,33 +1963,41 @@
         <v>54.4</v>
       </c>
       <c r="N2" s="5">
-        <f t="shared" ref="N2:N5" si="0">AVERAGE(J2:M2)</f>
+        <f>AVERAGE(J2:M2)</f>
         <v>56.524999999999999</v>
       </c>
-      <c r="O2" s="8">
-        <f t="shared" ref="O2:O5" si="1">N2/22</f>
+      <c r="O2" s="5">
+        <f>N2/1.12</f>
+        <v>50.468749999999993</v>
+      </c>
+      <c r="P2" s="8">
+        <f>N2/22</f>
         <v>2.5693181818181818</v>
       </c>
-      <c r="P2" s="5">
+      <c r="Q2" s="5">
         <v>39</v>
       </c>
-      <c r="Q2" s="5">
+      <c r="R2" s="5">
         <v>49.1</v>
       </c>
-      <c r="R2" s="5">
+      <c r="S2" s="5">
         <v>46.9</v>
       </c>
-      <c r="S2" s="5"/>
-      <c r="T2" s="5">
-        <f t="shared" ref="T2:T5" si="2">AVERAGE(P2:S2)</f>
+      <c r="T2" s="5"/>
+      <c r="U2" s="5">
+        <f t="shared" ref="U2:U5" si="0">AVERAGE(Q2:T2)</f>
         <v>45</v>
       </c>
-      <c r="U2" s="6">
-        <f>T2/22</f>
+      <c r="V2" s="5">
+        <f>U2/1.12</f>
+        <v>40.178571428571423</v>
+      </c>
+      <c r="W2" s="6">
+        <f>U2/22</f>
         <v>2.0454545454545454</v>
       </c>
     </row>
-    <row r="3" spans="1:21">
+    <row r="3" spans="1:23">
       <c r="A3" s="5">
         <v>0.6</v>
       </c>
@@ -2006,31 +2038,39 @@
         <v>50.1</v>
       </c>
       <c r="N3" s="5">
+        <f t="shared" ref="N3:N5" si="1">AVERAGE(J3:M3)</f>
+        <v>49.424999999999997</v>
+      </c>
+      <c r="O3" s="5">
+        <f t="shared" ref="O3:O5" si="2">N3/1.12</f>
+        <v>44.129464285714278</v>
+      </c>
+      <c r="P3" s="8">
+        <f>N3/22</f>
+        <v>2.2465909090909091</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>28.8</v>
+      </c>
+      <c r="R3" s="5">
+        <v>30</v>
+      </c>
+      <c r="S3" s="5"/>
+      <c r="T3" s="5"/>
+      <c r="U3" s="5">
         <f t="shared" si="0"/>
-        <v>49.424999999999997</v>
-      </c>
-      <c r="O3" s="8">
-        <f t="shared" si="1"/>
-        <v>2.2465909090909091</v>
-      </c>
-      <c r="P3" s="5">
-        <v>28.8</v>
-      </c>
-      <c r="Q3" s="5">
-        <v>30</v>
-      </c>
-      <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="5">
-        <f t="shared" si="2"/>
         <v>29.4</v>
       </c>
-      <c r="U3" s="6">
-        <f>T3/22</f>
+      <c r="V3" s="5">
+        <f t="shared" ref="V3:V5" si="3">U3/1.12</f>
+        <v>26.249999999999996</v>
+      </c>
+      <c r="W3" s="6">
+        <f>U3/22</f>
         <v>1.3363636363636362</v>
       </c>
     </row>
-    <row r="4" spans="1:21">
+    <row r="4" spans="1:23">
       <c r="A4" s="5">
         <v>0.9</v>
       </c>
@@ -2071,35 +2111,43 @@
         <v>49.3</v>
       </c>
       <c r="N4" s="5">
+        <f t="shared" si="1"/>
+        <v>52.400000000000006</v>
+      </c>
+      <c r="O4" s="5">
+        <f t="shared" si="2"/>
+        <v>46.785714285714285</v>
+      </c>
+      <c r="P4" s="8">
+        <f>N4/22</f>
+        <v>2.3818181818181823</v>
+      </c>
+      <c r="Q4" s="5">
+        <v>34.200000000000003</v>
+      </c>
+      <c r="R4" s="5">
+        <v>40.200000000000003</v>
+      </c>
+      <c r="S4" s="5">
+        <v>32.9</v>
+      </c>
+      <c r="T4" s="5">
+        <v>33.700000000000003</v>
+      </c>
+      <c r="U4" s="5">
         <f t="shared" si="0"/>
-        <v>52.400000000000006</v>
-      </c>
-      <c r="O4" s="8">
-        <f t="shared" si="1"/>
-        <v>2.3818181818181823</v>
-      </c>
-      <c r="P4" s="5">
-        <v>34.200000000000003</v>
-      </c>
-      <c r="Q4" s="5">
-        <v>40.200000000000003</v>
-      </c>
-      <c r="R4" s="5">
-        <v>32.9</v>
-      </c>
-      <c r="S4" s="5">
-        <v>33.700000000000003</v>
-      </c>
-      <c r="T4" s="5">
-        <f t="shared" si="2"/>
         <v>35.25</v>
       </c>
-      <c r="U4" s="6">
-        <f t="shared" ref="U4:U5" si="3">T4/22</f>
+      <c r="V4" s="5">
+        <f t="shared" si="3"/>
+        <v>31.473214285714281</v>
+      </c>
+      <c r="W4" s="6">
+        <f t="shared" ref="W4:W5" si="4">U4/22</f>
         <v>1.6022727272727273</v>
       </c>
     </row>
-    <row r="5" spans="1:21">
+    <row r="5" spans="1:23">
       <c r="A5" s="5">
         <v>0.9</v>
       </c>
@@ -2140,89 +2188,110 @@
         <v>55.4</v>
       </c>
       <c r="N5" s="5">
+        <f t="shared" si="1"/>
+        <v>53.524999999999999</v>
+      </c>
+      <c r="O5" s="5">
+        <f t="shared" si="2"/>
+        <v>47.790178571428562</v>
+      </c>
+      <c r="P5" s="8">
+        <f>N5/22</f>
+        <v>2.4329545454545456</v>
+      </c>
+      <c r="Q5" s="5">
+        <v>33.5</v>
+      </c>
+      <c r="R5" s="5">
+        <v>33.799999999999997</v>
+      </c>
+      <c r="S5" s="5"/>
+      <c r="T5" s="5"/>
+      <c r="U5" s="5">
         <f t="shared" si="0"/>
-        <v>53.524999999999999</v>
-      </c>
-      <c r="O5" s="8">
-        <f t="shared" si="1"/>
-        <v>2.4329545454545456</v>
-      </c>
-      <c r="P5" s="5">
-        <v>33.5</v>
-      </c>
-      <c r="Q5" s="5">
-        <v>33.799999999999997</v>
-      </c>
-      <c r="R5" s="5"/>
-      <c r="S5" s="5"/>
-      <c r="T5" s="5">
-        <f t="shared" si="2"/>
         <v>33.65</v>
       </c>
-      <c r="U5" s="6">
+      <c r="V5" s="5">
         <f t="shared" si="3"/>
+        <v>30.044642857142854</v>
+      </c>
+      <c r="W5" s="6">
+        <f t="shared" si="4"/>
         <v>1.5295454545454545</v>
       </c>
     </row>
-    <row r="6" spans="1:21">
-      <c r="O6" s="8">
+    <row r="6" spans="1:23">
+      <c r="J6" s="9"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="9">
         <f>AVERAGE(O2:O5)</f>
+        <v>47.293526785714278</v>
+      </c>
+      <c r="P6" s="8">
+        <f>AVERAGE(P2:P5)</f>
         <v>2.407670454545455</v>
       </c>
-      <c r="U6" s="8">
-        <f>AVERAGE(U2:U5)</f>
+      <c r="V6" s="8">
+        <f>AVERAGE(V2:V5)</f>
+        <v>31.986607142857139</v>
+      </c>
+      <c r="W6" s="8">
+        <f>AVERAGE(W2:W5)</f>
         <v>1.6284090909090909</v>
       </c>
     </row>
-    <row r="7" spans="1:21">
+    <row r="7" spans="1:23">
       <c r="B7" s="18"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
-      <c r="O7" s="8">
-        <f>22*O6</f>
+      <c r="J7" s="5"/>
+      <c r="O7" s="5"/>
+      <c r="P7" s="8">
+        <f>22*P6</f>
         <v>52.968750000000014</v>
       </c>
-      <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
       <c r="S7" s="8"/>
       <c r="T7" s="8"/>
-      <c r="U7" s="8">
-        <f t="shared" ref="U7" si="4">22*U6</f>
+      <c r="U7" s="8"/>
+      <c r="V7" s="8"/>
+      <c r="W7" s="8">
+        <f>22*W6</f>
         <v>35.825000000000003</v>
       </c>
     </row>
-    <row r="8" spans="1:21">
+    <row r="8" spans="1:23">
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
       <c r="D8" s="12"/>
       <c r="E8" s="6"/>
     </row>
-    <row r="9" spans="1:21">
+    <row r="9" spans="1:23">
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
       <c r="D9" s="12"/>
       <c r="E9" s="6"/>
     </row>
-    <row r="10" spans="1:21">
+    <row r="10" spans="1:23">
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
       <c r="D10" s="12"/>
       <c r="E10" s="6"/>
     </row>
-    <row r="11" spans="1:21">
+    <row r="11" spans="1:23">
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
       <c r="D11" s="12"/>
       <c r="E11" s="6"/>
     </row>
-    <row r="12" spans="1:21">
+    <row r="12" spans="1:23">
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
       <c r="D12" s="12"/>
       <c r="E12" s="6"/>
     </row>
-    <row r="13" spans="1:21">
+    <row r="13" spans="1:23">
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
       <c r="D13" s="12"/>

</xml_diff>